<commit_message>
Add apprenticeship skill configs
</commit_message>
<xml_diff>
--- a/jyx2/Assets/Mods/jshyl/Configs/武功.xlsx
+++ b/jyx2/Assets/Mods/jshyl/Configs/武功.xlsx
@@ -560,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G205"/>
+  <dimension ref="A1:G210"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="14.26953125" customWidth="1" style="11" min="3" max="3"/>
@@ -4256,29 +4256,164 @@
       <c r="G204" s="2" t="n"/>
     </row>
     <row r="205">
-      <c r="A205" t="n">
+      <c r="A205" s="0" t="n">
         <v>205</v>
       </c>
-      <c r="B205" t="inlineStr">
+      <c r="B205" s="0" t="inlineStr">
         <is>
           <t>独孤九剑</t>
         </is>
       </c>
-      <c r="C205" t="n">
-        <v>0</v>
-      </c>
-      <c r="D205" t="n">
+      <c r="C205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D205" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="E205" t="n">
+      <c r="E205" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F205" t="n">
-        <v>0</v>
-      </c>
-      <c r="G205" t="inlineStr">
+      <c r="F205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G205" s="0" t="inlineStr">
         <is>
           <t>100,3,1,0,0|150,3,1,0,0|200,3,1,0,0|250,5,2,0,0|300,5,2,0,0|350,5,2,0,0|400,7,3,0,0|450,7,3,0,0|500,7,3,0,0|800,7,3,0,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="0" t="n">
+        <v>206</v>
+      </c>
+      <c r="B206" s="0" t="inlineStr">
+        <is>
+          <t>七弦无形剑</t>
+        </is>
+      </c>
+      <c r="C206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D206" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E206" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="F206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G206" s="0" t="inlineStr">
+        <is>
+          <t>25,3,0,0,0|50,3,0,0,0|75,3,0,0,0|100,4,0,0,0|125,4,0,0,0|150,4,0,0,0|175,5,0,0,0|200,5,0,0,0|225,5,0,0,0|400,6,0,0,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="0" t="n">
+        <v>207</v>
+      </c>
+      <c r="B207" s="0" t="inlineStr">
+        <is>
+          <t>回风舞柳剑</t>
+        </is>
+      </c>
+      <c r="C207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D207" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E207" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G207" s="0" t="inlineStr">
+        <is>
+          <t>50,2,0,0,0|70,2,0,0,0|80,2,0,0,0|90,3,1,0,0|100,3,1,0,0|110,3,1,0,0|120,4,1,0,0|130,4,2,0,0|140,4,2,0,0|300,5,2,0,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="0" t="n">
+        <v>208</v>
+      </c>
+      <c r="B208" s="0" t="inlineStr">
+        <is>
+          <t>如影随形腿</t>
+        </is>
+      </c>
+      <c r="C208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D208" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E208" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G208" s="0" t="inlineStr">
+        <is>
+          <t>20,1,0,0,0|25,2,0,0,0|30,3,0,0,0|40,4,0,0,0|50,4,0,0,0|55,4,0,0,0|60,4,0,0,0|65,4,0,0,0|70,4,0,0,0|200,4,0,0,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="0" t="n">
+        <v>209</v>
+      </c>
+      <c r="B209" s="0" t="inlineStr">
+        <is>
+          <t>飞沙走石刀</t>
+        </is>
+      </c>
+      <c r="C209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E209" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="F209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G209" s="0" t="inlineStr">
+        <is>
+          <t>30,1,0,0,0|45,1,0,0,0|60,1,0,0,0|70,1,0,0,0|80,2,0,0,0|90,2,0,0,0|100,2,0,0,0|110,2,0,0,0|120,3,0,0,0|250,3,0,0,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="0" t="n">
+        <v>210</v>
+      </c>
+      <c r="B210" s="0" t="inlineStr">
+        <is>
+          <t>大风云飞掌</t>
+        </is>
+      </c>
+      <c r="C210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E210" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="F210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G210" s="0" t="inlineStr">
+        <is>
+          <t>20,1,0,0,0|40,1,0,0,0|60,2,0,0,0|80,2,0,0,0|100,3,0,0,0|120,3,0,0,0|140,4,0,0,0|160,4,0,0,0|180,5,0,0,0|300,5,0,0,0</t>
         </is>
       </c>
     </row>

</xml_diff>